<commit_message>
Add AI Use Cases sheet to Excel workbook with 46 use cases
New sheet covers 7 categories with example prompts and value descriptions:
- Data Exploration & Understanding (6 use cases)
- Statistical Analysis & Diagnostics (7 use cases)
- Model Development Support (7 use cases)
- Model Validation & Monitoring (6 use cases)
- Regulatory & Compliance (5 use cases)
- Data Engineering & Operations (5 use cases)
- Business Intelligence & Reporting (5 use cases)
- Advanced Analytics & ML (5 use cases)

Each use case includes description, example prompt to agent, data sources
used, and value to the modeler.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNcNPd22aFMjdQZijhWxwY
</commit_message>
<xml_diff>
--- a/data/generated/credit_bureau_data_dictionaries.xlsx
+++ b/data/generated/credit_bureau_data_dictionaries.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Credit Card" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Mortgage" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Personal Loan" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="AI Use Cases" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Experian'!$A$1:$AN$26</definedName>
@@ -40,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +88,31 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -203,6 +227,12 @@
         <bgColor rgb="00EF6C00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0FE"/>
+        <bgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -230,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -306,6 +336,22 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -22329,6 +22375,1815 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E7D32"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>AI Agent Use Cases for Credit Risk Modeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Comprehensive catalog of how the AI agent helps modelers across the credit risk lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Use Case</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Example Prompt to Agent</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Data Sources Used</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Value to Modeler</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n"/>
+      <c r="C5" s="31" t="n"/>
+      <c r="D5" s="31" t="n"/>
+      <c r="E5" s="31" t="n"/>
+      <c r="F5" s="31" t="n"/>
+      <c r="G5" s="31" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Attribute Lookup</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Look up any attribute by name or keyword and get its full definition, valid ranges, special values, data type, and which bureau/source it comes from.</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>What is REVOL_UTIL? What are its valid values and what do the special codes mean?</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Experian, Equifax, TransUnion, LexisNexis, Internal</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Eliminates time spent searching through PDF documentation or asking senior analysts. Instant, accurate answers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Attribute Comparison Across Bureaus</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Compare similar attributes across Experian, Equifax, and TransUnion to understand differences in naming, ranges, and definitions.</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Compare revolving utilization across all three bureaus — how do they differ in definition and typical ranges?</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Experian, Equifax, TransUnion</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Prevents errors when merging multi-bureau data. Clarifies subtle definitional differences that affect model performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Special Value Decoder</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Explain what each special/sentinel value means for an attribute (e.g., -1 = No Data, -5 = No Hit) and how to handle them in modeling.</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>What do the negative values in EFX_BEACON_5 mean and how should I treat them in my model?</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Prevents silent data errors — miscoding a -1 (thin file) as a real value corrupts model training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Segment-Based Attribute Discovery</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Find all attributes in a segment (e.g., delinquency, utilization, scores) across all sources to see the full landscape.</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>Show me all delinquency-related attributes across all bureaus and internal data.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Accelerates feature selection by surfacing all available features in a risk dimension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Data Type &amp; Range Validation Guide</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>For any attribute, get the expected data type, valid range, and flag values outside range as potential data quality issues.</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>What is the expected range for NUM_30DPD_12M and what would be considered an outlier?</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Catches data quality issues early before they propagate into model development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Data Exploration &amp; Understanding</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>New Modeler Onboarding</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Walk a new modeler through the complete attribute landscape — what each source provides, key differences, and where to start.</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>I'm new to credit modeling. Walk me through what data we have from each bureau and what the internal data covers.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Reduces onboarding time from weeks to hours. New modelers become productive immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="31" t="n"/>
+      <c r="G12" s="31" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Univariate Statistics Summary</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Get min, max, mean, median, and standard deviation for any attribute, broken out by portfolio.</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>What are the descriptive statistics for FICO Score V2 across all four portfolios?</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Instant statistical profiling without writing code or running queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>KS Statistic Interpretation</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Explain the Kolmogorov-Smirnov (KS) statistic for each attribute, what it measures, and rank attributes by discriminatory power.</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>Which attributes have the highest KS for the auto loan portfolio? What does a KS of 42 mean?</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Prioritizes features by how well they separate good from bad — essential for scorecard development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>PSI Monitoring &amp; Drift Detection</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Check Population Stability Index for each attribute to detect distribution shifts between development and recent data.</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Which attributes show PSI above 0.10 for personal loans? Should I be concerned about population drift?</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Early warning system for model degradation. Attributes with high PSI may need recalibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Feature Importance Ranking</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Rank all attributes by their importance to the target variable for a specific portfolio.</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Rank the top 20 most important attributes for predicting 90+ DPD in the credit card portfolio.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Guides feature selection and helps modelers focus on high-value attributes first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Cross-Portfolio Comparison</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Compare how an attribute behaves differently across portfolios (auto vs. credit card vs. mortgage vs. personal loan).</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>How does revolving utilization differ in importance and distribution between auto loans and credit cards?</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Reveals portfolio-specific patterns that inform whether to build separate models or a single model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Distribution Profiling</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Describe the shape of an attribute's distribution (skewed, bimodal, zero-inflated) and implications for modeling.</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>Describe the distribution of NUM_COLLECTIONS — is it zero-inflated? How should I transform it?</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Informs transformation decisions (log, WoE binning) and whether to treat as continuous or categorical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>Statistical Analysis &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Outlier &amp; Anomaly Identification</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Flag records or attribute values that fall outside expected ranges or show suspicious patterns.</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>Are there any records in the auto loan data where FICO is above 850 or below 300? What about negative balances?</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Generated Data</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Data quality gate before model development — catch impossible values before they bias the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="31" t="n"/>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Feature Selection Guidance</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Recommend which features to include in a model based on KS, importance, correlation, and practical considerations.</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>I'm building an auto loan scorecard. Which 15 features should I start with and why?</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Expert-level feature selection advice that balances statistical power with interpretability and regulatory requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Multicollinearity Assessment</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Identify attributes likely to be highly correlated (e.g., multiple score versions, overlapping balance measures) and recommend which to keep.</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>FICOCV2 and FICOCV3 seem similar — should I include both in my model? What about all the balance attributes?</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Prevents multicollinearity issues that inflate variance and make coefficients unstable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Target Variable Selection</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Compare available target definitions (30 DPD, 60 DPD, 90 DPD, charge-off) and recommend the best for a given use case.</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>Should I use 60+ DPD at 12 months or 90+ DPD at 24 months as my target for an auto loan PD model?</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Aligns model objective with business need and regulatory requirements (Basel, CECL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Missing Data Strategy</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Analyze missing rates per attribute and recommend imputation strategies (mean, median, WoE bin, separate indicator).</t>
+        </is>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>Which attributes have high missing rates for mortgage? What imputation approach do you recommend for each?</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Prevents information loss from naive imputation and ensures special values are handled correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>WoE / IV Binning Guidance</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Advise on Weight of Evidence binning strategies for each attribute type (continuous, categorical, zero-inflated).</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>How should I bin OLDEST_TL_MTHS for WoE analysis? What bin boundaries would you recommend?</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Accelerates the tedious binning process with informed starting points based on attribute characteristics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Reject Inference Support</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Identify which attributes are available at application (pre-decision) vs. only post-booking for reject inference.</t>
+        </is>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>Which internal attributes are available at application time and which are only available after booking?</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Internal, Performance</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Ensures reject inference uses only through-the-door attributes, preventing data leakage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Model Development Support</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard Reason Code Mapping</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Map model features to human-readable adverse action reason codes required under ECOA/FCRA.</t>
+        </is>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>If REVOL_UTIL is a top driver of decline, what adverse action reason code should we assign?</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Regulatory compliance — every decline must provide specific, accurate reasons to the applicant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="n"/>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="31" t="n"/>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="31" t="n"/>
+      <c r="G28" s="31" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Model Performance Benchmarking</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Compare expected KS and feature importance against actual model performance to identify potential issues.</t>
+        </is>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>My auto loan model has a KS of 35 — is that good? How does it compare to what we'd expect from the feature set?</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Reality check on model performance — is the model extracting expected information from the features?</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Population Stability Monitoring</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Monitor PSI trends across all features to detect when the applicant population has shifted.</t>
+        </is>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>Run a PSI check across all features for the personal loan portfolio. Which ones are drifting?</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Proactive model risk management — detect drift before it degrades model performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Feature Contribution Analysis</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Analyze whether each feature's importance has changed over time compared to development.</t>
+        </is>
+      </c>
+      <c r="E31" s="33" t="inlineStr">
+        <is>
+          <t>Has the importance of credit scores decreased relative to delinquency counts in recent data?</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Detects structural changes in the relationship between features and default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Challenger Model Support</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Identify new features or alternative data sources that could improve an existing model.</t>
+        </is>
+      </c>
+      <c r="E32" s="33" t="inlineStr">
+        <is>
+          <t>We have a FICO-only auto model. What LexisNexis or CreditVision features could add lift?</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>LexisNexis, TransUnion CreditVision</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Guides challenger model development with data-driven feature recommendations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Vintage Analysis Support</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Use origination dates and performance windows to structure vintage-based model monitoring.</t>
+        </is>
+      </c>
+      <c r="E33" s="33" t="inlineStr">
+        <is>
+          <t>How should I set up vintage cohorts for monitoring the mortgage portfolio's 90 DPD rate?</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Structures the performance monitoring framework to catch deterioration by origination cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>Model Validation &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Back-Testing Validation</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Compare model predictions against actual outcomes using the performance data.</t>
+        </is>
+      </c>
+      <c r="E34" s="33" t="inlineStr">
+        <is>
+          <t>Show me the actual 90+ DPD rate by FICO decile for the auto loan portfolio.</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Performance + Generated Data</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Validates that the model rank-orders risk correctly across the score range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="n"/>
+      <c r="C35" s="31" t="n"/>
+      <c r="D35" s="31" t="n"/>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="31" t="n"/>
+      <c r="G35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Fair Lending Analysis Support</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Identify attributes that may serve as proxies for prohibited bases (race, gender, age) and flag for disparate impact testing.</t>
+        </is>
+      </c>
+      <c r="E36" s="33" t="inlineStr">
+        <is>
+          <t>Which LexisNexis attributes could be proxies for protected classes? Should we exclude any from a fair lending perspective?</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>LexisNexis, Internal</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Proactive fair lending risk identification before model goes to compliance review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Model Documentation Generation</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Generate model development documentation sections including feature definitions, data sources, and summary statistics.</t>
+        </is>
+      </c>
+      <c r="E37" s="33" t="inlineStr">
+        <is>
+          <t>Generate the 'Data Description' section for my model document covering all Experian attributes used.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Automates the most tedious part of MRM documentation — accurate, consistent, and audit-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>CECL / IFRS 9 Feature Mapping</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Map attributes to CECL lifetime loss estimation requirements — PD, LGD, EAD components.</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>Which attributes best predict loss given default for the mortgage portfolio? Map them to CECL requirements.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Performance</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Bridges the gap between data dictionary and regulatory model requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>SR 11-7 / OCC 2011-12 Compliance Check</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Verify that model features, data sources, and performance metrics align with regulatory guidance on model risk management.</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>Does our feature set meet SR 11-7 expectations for conceptual soundness? Are there any gaps?</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Ensures the model passes MRM review by checking features against regulatory expectations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>FCRA Permissible Purpose Verification</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Verify that each data source and attribute is used within its permissible purpose under FCRA.</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>Can I use LexisNexis criminal records in an auto loan origination model? What are the FCRA implications?</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>LexisNexis, All Sources</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Prevents compliance violations from using data outside permissible purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="n"/>
+      <c r="C41" s="31" t="n"/>
+      <c r="D41" s="31" t="n"/>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="31" t="n"/>
+      <c r="G41" s="31" t="n"/>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>ETL Validation Rules Generation</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Generate data validation rules (range checks, type checks, special value handling) for ETL pipelines.</t>
+        </is>
+      </c>
+      <c r="E42" s="33" t="inlineStr">
+        <is>
+          <t>Generate validation rules for all Equifax attributes — range checks, null handling, and special value mapping.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Automates creation of data quality checks for production ETL pipelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B43" s="32" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Data Mapping Across Sources</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Create a crosswalk between similar attributes across bureaus for multi-bureau data integration.</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>Create a mapping table showing equivalent attributes across Experian, Equifax, and TransUnion.</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Experian, Equifax, TransUnion</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Enables consistent multi-bureau feature engineering without manual cross-referencing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Schema Documentation</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Generate database schema documentation including column names, types, constraints, and descriptions.</t>
+        </is>
+      </c>
+      <c r="E44" s="33" t="inlineStr">
+        <is>
+          <t>Generate a CREATE TABLE DDL statement for the auto loan feature table with all attribute definitions as comments.</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Speeds up data warehouse setup with accurate, documented schemas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="B45" s="32" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Data Quality Report Generation</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Produce a comprehensive data quality report covering completeness, validity, and distribution checks.</t>
+        </is>
+      </c>
+      <c r="E45" s="33" t="inlineStr">
+        <is>
+          <t>Generate a data quality report for the personal loan portfolio covering all 107 attributes.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Automated QA reporting that would otherwise take analysts days to compile manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B46" s="32" t="inlineStr">
+        <is>
+          <t>Data Engineering &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Feature Store Documentation</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Document features for a feature store including metadata, lineage, freshness, and usage.</t>
+        </is>
+      </c>
+      <c r="E46" s="33" t="inlineStr">
+        <is>
+          <t>Document all TransUnion CreditVision attributes for our feature store — include refresh frequency and downstream models.</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Enables feature reuse across models and teams with proper governance metadata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="30" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="B47" s="31" t="n"/>
+      <c r="C47" s="31" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="31" t="n"/>
+      <c r="F47" s="31" t="n"/>
+      <c r="G47" s="31" t="n"/>
+    </row>
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio Risk Profile</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Generate a risk profile summary for any portfolio showing key risk indicators and their distributions.</t>
+        </is>
+      </c>
+      <c r="E48" s="33" t="inlineStr">
+        <is>
+          <t>Give me a risk profile of the auto loan portfolio — what does the typical applicant look like across all key metrics?</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>All Sources + Generated Data</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Instant portfolio-level insights for management reporting and strategy discussions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Segment Comparison Dashboard</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Compare risk characteristics across segments (e.g., prime vs. subprime, new vs. existing customers).</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="inlineStr">
+        <is>
+          <t>Compare the risk profile of existing customers vs. new customers applying for personal loans.</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Internal + All Sources</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Data-driven segmentation insights for pricing and policy decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Trend Analysis &amp; Early Warning</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Identify attributes showing adverse trends that may signal portfolio deterioration.</t>
+        </is>
+      </c>
+      <c r="E50" s="33" t="inlineStr">
+        <is>
+          <t>Which attributes in the credit card portfolio show worsening trends based on PSI and distribution shifts?</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Early warning system for portfolio managers to take preemptive action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B51" s="32" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Executive Summary Generation</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Create non-technical summaries of model features and performance for executive stakeholders.</t>
+        </is>
+      </c>
+      <c r="E51" s="33" t="inlineStr">
+        <is>
+          <t>Summarize our auto loan model's key risk drivers in plain English for the Chief Risk Officer.</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Bridges the gap between technical model output and business-level understanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="B52" s="32" t="inlineStr">
+        <is>
+          <t>Business Intelligence &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Loss Forecasting Support</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Use performance data and feature distributions to support loss forecasting and stress testing.</t>
+        </is>
+      </c>
+      <c r="E52" s="33" t="inlineStr">
+        <is>
+          <t>Based on current portfolio composition, what loss rate should we expect for the personal loan book?</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Performance + All Sources</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Connects bottom-up feature analysis to top-down loss forecasting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="30" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="B53" s="31" t="n"/>
+      <c r="C53" s="31" t="n"/>
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="31" t="n"/>
+      <c r="F53" s="31" t="n"/>
+      <c r="G53" s="31" t="n"/>
+    </row>
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="B54" s="32" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Alternative Data Assessment</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Evaluate the incremental value of LexisNexis alternative data over traditional bureau data.</t>
+        </is>
+      </c>
+      <c r="E54" s="33" t="inlineStr">
+        <is>
+          <t>How much lift would adding LexisNexis RiskView and address stability provide over bureau scores alone for thin-file applicants?</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>LexisNexis + Bureau Sources</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Quantifies the business case for purchasing additional data sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="60" customHeight="1">
+      <c r="A55" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="B55" s="32" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Feature Engineering Ideas</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Suggest derived features and interaction terms based on the raw attributes available.</t>
+        </is>
+      </c>
+      <c r="E55" s="33" t="inlineStr">
+        <is>
+          <t>What feature interactions or ratios should I create from the bureau and internal data for a personal loan model?</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Accelerates feature engineering with domain-informed suggestions (e.g., payment-to-income ratios, utilization trends).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="60" customHeight="1">
+      <c r="A56" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B56" s="32" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>ML vs. Scorecard Feature Selection</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Compare feature recommendations for a traditional logistic regression scorecard vs. a gradient boosted model.</t>
+        </is>
+      </c>
+      <c r="E56" s="33" t="inlineStr">
+        <is>
+          <t>I'm building both a scorecard and an XGBoost model for auto loans — how should feature selection differ between them?</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Tailored feature strategies for different modeling approaches — scorecards need fewer, interpretable features while ML can use more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Trended Data Strategy</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Advise on using TransUnion CreditVision trended data features (payment velocity, balance trends) effectively.</t>
+        </is>
+      </c>
+      <c r="E57" s="33" t="inlineStr">
+        <is>
+          <t>How should I incorporate CreditVision payment velocity and balance trend into my credit card model?</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>TransUnion CreditVision</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Unlocks value from trended data — a newer data dimension many modelers underutilize.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B58" s="32" t="inlineStr">
+        <is>
+          <t>Advanced Analytics &amp; ML</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Model Explainability Support</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Help interpret model outputs by connecting predictions back to individual feature contributions and definitions.</t>
+        </is>
+      </c>
+      <c r="E58" s="33" t="inlineStr">
+        <is>
+          <t>A customer was declined — explain which features drove the decision and what each one means in plain language.</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>All Sources</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Supports SHAP/LIME explainability by providing human-readable context for each feature contribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Total: 46 use cases across 8 categories</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update SR 11-7 reference to SR 26-3
The Fed's model risk management guidance was superseded by SR 26-3.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WNcNPd22aFMjdQZijhWxwY
</commit_message>
<xml_diff>
--- a/data/generated/credit_bureau_data_dictionaries.xlsx
+++ b/data/generated/credit_bureau_data_dictionaries.xlsx
@@ -23536,7 +23536,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>SR 11-7 / OCC 2011-12 Compliance Check</t>
+          <t>SR 26-3 / OCC 2011-12 Compliance Check</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -23546,7 +23546,7 @@
       </c>
       <c r="E39" s="33" t="inlineStr">
         <is>
-          <t>Does our feature set meet SR 11-7 expectations for conceptual soundness? Are there any gaps?</t>
+          <t>Does our feature set meet SR 26-3 expectations for conceptual soundness? Are there any gaps?</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Ensures the model passes MRM review by checking features against regulatory expectations.</t>
+          <t>Ensures the model passes MRM review by checking features against SR 26-3 regulatory expectations.</t>
         </is>
       </c>
     </row>

</xml_diff>